<commit_message>
Regenerated datasets to including a running_quarter variable
</commit_message>
<xml_diff>
--- a/Data/Final Data/No Controls/State/STATE_NO_CONTROLS_VIC_NSW_Median_Rent.xlsx
+++ b/Data/Final Data/No Controls/State/STATE_NO_CONTROLS_VIC_NSW_Median_Rent.xlsx
@@ -361,7 +361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -409,6 +409,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -441,6 +446,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -473,6 +481,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -505,6 +516,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,6 +551,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -569,6 +586,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -601,6 +621,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -633,6 +656,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -665,6 +691,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -697,6 +726,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -729,6 +761,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -761,6 +796,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -793,6 +831,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -825,6 +866,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -857,6 +901,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -889,6 +936,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -921,6 +971,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -953,6 +1006,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -985,6 +1041,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1017,6 +1076,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1049,6 +1111,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1081,6 +1146,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1113,6 +1181,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1145,6 +1216,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1177,6 +1251,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1209,6 +1286,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1241,6 +1321,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1273,6 +1356,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1305,6 +1391,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1337,6 +1426,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1369,6 +1461,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1401,6 +1496,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1433,6 +1531,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1465,6 +1566,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1497,6 +1601,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1529,6 +1636,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1561,6 +1671,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1593,6 +1706,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1624,6 +1740,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1633,7 +1752,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -1681,6 +1800,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1713,6 +1837,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1745,6 +1872,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1777,6 +1907,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1809,6 +1942,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1841,6 +1977,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1873,6 +2012,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1905,6 +2047,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1937,6 +2082,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1969,6 +2117,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2001,6 +2152,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2033,6 +2187,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2065,6 +2222,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2097,6 +2257,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2129,6 +2292,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2161,6 +2327,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2193,6 +2362,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2225,6 +2397,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2257,6 +2432,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2289,6 +2467,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2321,6 +2502,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2353,6 +2537,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2385,6 +2572,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2417,6 +2607,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2449,6 +2642,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2481,6 +2677,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2513,6 +2712,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2545,6 +2747,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2577,6 +2782,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2609,6 +2817,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2641,6 +2852,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2673,6 +2887,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2705,6 +2922,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2737,6 +2957,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2769,6 +2992,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2801,6 +3027,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2833,6 +3062,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2865,6 +3097,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2896,6 +3131,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2905,7 +3143,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -2953,6 +3191,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2985,6 +3228,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3017,6 +3263,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3049,6 +3298,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3081,6 +3333,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3113,6 +3368,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3145,6 +3403,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3177,6 +3438,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3209,6 +3473,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3241,6 +3508,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3273,6 +3543,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3305,6 +3578,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3337,6 +3613,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3369,6 +3648,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3401,6 +3683,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3433,6 +3718,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3465,6 +3753,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3497,6 +3788,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3529,6 +3823,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3561,6 +3858,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3593,6 +3893,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3625,6 +3928,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3657,6 +3963,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3689,6 +3998,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3721,6 +4033,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3753,6 +4068,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3785,6 +4103,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3817,6 +4138,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3849,6 +4173,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3881,6 +4208,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3913,6 +4243,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3945,6 +4278,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3977,6 +4313,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4009,6 +4348,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4041,6 +4383,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4073,6 +4418,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4105,6 +4453,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4137,6 +4488,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4168,6 +4522,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -4177,7 +4534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -4225,6 +4582,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4257,6 +4619,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4289,6 +4654,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4321,6 +4689,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4353,6 +4724,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4385,6 +4759,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4417,6 +4794,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4449,6 +4829,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4481,6 +4864,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4513,6 +4899,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4545,6 +4934,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4577,6 +4969,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4609,6 +5004,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4641,6 +5039,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4673,6 +5074,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4705,6 +5109,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4737,6 +5144,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4769,6 +5179,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4801,6 +5214,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4833,6 +5249,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4865,6 +5284,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4897,6 +5319,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4929,6 +5354,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4961,6 +5389,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4993,6 +5424,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5025,6 +5459,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5057,6 +5494,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5089,6 +5529,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5121,6 +5564,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5153,6 +5599,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5185,6 +5634,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5217,6 +5669,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5249,6 +5704,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5281,6 +5739,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5313,6 +5774,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5345,6 +5809,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5377,6 +5844,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5409,6 +5879,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5440,6 +5913,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -5449,7 +5925,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -5497,6 +5973,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5529,6 +6010,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5561,6 +6045,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5593,6 +6080,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5625,6 +6115,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5657,6 +6150,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -5689,6 +6185,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5721,6 +6220,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5753,6 +6255,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5785,6 +6290,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5817,6 +6325,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5849,6 +6360,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5881,6 +6395,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5913,6 +6430,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5945,6 +6465,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5977,6 +6500,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6009,6 +6535,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6041,6 +6570,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6073,6 +6605,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6105,6 +6640,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6137,6 +6675,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6169,6 +6710,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6201,6 +6745,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6233,6 +6780,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6265,6 +6815,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6297,6 +6850,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6329,6 +6885,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6361,6 +6920,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6393,6 +6955,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6425,6 +6990,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -6457,6 +7025,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -6489,6 +7060,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -6521,6 +7095,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -6553,6 +7130,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -6585,6 +7165,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -6617,6 +7200,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -6649,6 +7235,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -6681,6 +7270,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -6712,6 +7304,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -6721,7 +7316,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -6769,6 +7364,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6801,6 +7401,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6833,6 +7436,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6865,6 +7471,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6897,6 +7506,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6929,6 +7541,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6961,6 +7576,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6993,6 +7611,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7025,6 +7646,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7057,6 +7681,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7089,6 +7716,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7121,6 +7751,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7153,6 +7786,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7185,6 +7821,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7217,6 +7856,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7249,6 +7891,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7281,6 +7926,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7313,6 +7961,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7345,6 +7996,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7377,6 +8031,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7409,6 +8066,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7441,6 +8101,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7473,6 +8136,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7505,6 +8171,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -7537,6 +8206,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -7569,6 +8241,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -7601,6 +8276,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -7633,6 +8311,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -7665,6 +8346,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -7697,6 +8381,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7729,6 +8416,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7761,6 +8451,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7793,6 +8486,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7825,6 +8521,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7857,6 +8556,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7889,6 +8591,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7921,6 +8626,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7953,6 +8661,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7984,6 +8695,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -7993,7 +8707,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="7" max="7" width="20.7109375" style="2" customWidth="1"/>
@@ -8041,6 +8755,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Running_Quarter</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8073,6 +8792,9 @@
       <c r="H2" s="2">
         <v>43465</v>
       </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8105,6 +8827,9 @@
       <c r="H3" s="2">
         <v>43830</v>
       </c>
+      <c r="I3">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8137,6 +8862,9 @@
       <c r="H4" s="2">
         <v>44196</v>
       </c>
+      <c r="I4">
+        <v>12</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8169,6 +8897,9 @@
       <c r="H5" s="2">
         <v>44561</v>
       </c>
+      <c r="I5">
+        <v>16</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8201,6 +8932,9 @@
       <c r="H6" s="2">
         <v>43281</v>
       </c>
+      <c r="I6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8233,6 +8967,9 @@
       <c r="H7" s="2">
         <v>43646</v>
       </c>
+      <c r="I7">
+        <v>6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8265,6 +9002,9 @@
       <c r="H8" s="2">
         <v>44012</v>
       </c>
+      <c r="I8">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8297,6 +9037,9 @@
       <c r="H9" s="2">
         <v>44377</v>
       </c>
+      <c r="I9">
+        <v>14</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8329,6 +9072,9 @@
       <c r="H10" s="2">
         <v>44742</v>
       </c>
+      <c r="I10">
+        <v>18</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8361,6 +9107,9 @@
       <c r="H11" s="2">
         <v>43190</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8393,6 +9142,9 @@
       <c r="H12" s="2">
         <v>43555</v>
       </c>
+      <c r="I12">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8425,6 +9177,9 @@
       <c r="H13" s="2">
         <v>43921</v>
       </c>
+      <c r="I13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8457,6 +9212,9 @@
       <c r="H14" s="2">
         <v>44286</v>
       </c>
+      <c r="I14">
+        <v>13</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8489,6 +9247,9 @@
       <c r="H15" s="2">
         <v>44651</v>
       </c>
+      <c r="I15">
+        <v>17</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8521,6 +9282,9 @@
       <c r="H16" s="2">
         <v>43373</v>
       </c>
+      <c r="I16">
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8553,6 +9317,9 @@
       <c r="H17" s="2">
         <v>43738</v>
       </c>
+      <c r="I17">
+        <v>7</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8585,6 +9352,9 @@
       <c r="H18" s="2">
         <v>44104</v>
       </c>
+      <c r="I18">
+        <v>11</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8617,6 +9387,9 @@
       <c r="H19" s="2">
         <v>44469</v>
       </c>
+      <c r="I19">
+        <v>15</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8649,6 +9422,9 @@
       <c r="H20" s="2">
         <v>44834</v>
       </c>
+      <c r="I20">
+        <v>19</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8681,6 +9457,9 @@
       <c r="H21" s="2">
         <v>43190</v>
       </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8713,6 +9492,9 @@
       <c r="H22" s="2">
         <v>43281</v>
       </c>
+      <c r="I22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8745,6 +9527,9 @@
       <c r="H23" s="2">
         <v>43373</v>
       </c>
+      <c r="I23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8777,6 +9562,9 @@
       <c r="H24" s="2">
         <v>43465</v>
       </c>
+      <c r="I24">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8809,6 +9597,9 @@
       <c r="H25" s="2">
         <v>43555</v>
       </c>
+      <c r="I25">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8841,6 +9632,9 @@
       <c r="H26" s="2">
         <v>43646</v>
       </c>
+      <c r="I26">
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8873,6 +9667,9 @@
       <c r="H27" s="2">
         <v>43738</v>
       </c>
+      <c r="I27">
+        <v>7</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8905,6 +9702,9 @@
       <c r="H28" s="2">
         <v>43830</v>
       </c>
+      <c r="I28">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8937,6 +9737,9 @@
       <c r="H29" s="2">
         <v>43921</v>
       </c>
+      <c r="I29">
+        <v>9</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8969,6 +9772,9 @@
       <c r="H30" s="2">
         <v>44012</v>
       </c>
+      <c r="I30">
+        <v>10</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9001,6 +9807,9 @@
       <c r="H31" s="2">
         <v>44104</v>
       </c>
+      <c r="I31">
+        <v>11</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9033,6 +9842,9 @@
       <c r="H32" s="2">
         <v>44196</v>
       </c>
+      <c r="I32">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9065,6 +9877,9 @@
       <c r="H33" s="2">
         <v>44286</v>
       </c>
+      <c r="I33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9097,6 +9912,9 @@
       <c r="H34" s="2">
         <v>44377</v>
       </c>
+      <c r="I34">
+        <v>14</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9129,6 +9947,9 @@
       <c r="H35" s="2">
         <v>44469</v>
       </c>
+      <c r="I35">
+        <v>15</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9161,6 +9982,9 @@
       <c r="H36" s="2">
         <v>44561</v>
       </c>
+      <c r="I36">
+        <v>16</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9193,6 +10017,9 @@
       <c r="H37" s="2">
         <v>44651</v>
       </c>
+      <c r="I37">
+        <v>17</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9225,6 +10052,9 @@
       <c r="H38" s="2">
         <v>44742</v>
       </c>
+      <c r="I38">
+        <v>18</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9256,6 +10086,9 @@
       </c>
       <c r="H39" s="2">
         <v>44834</v>
+      </c>
+      <c r="I39">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerated datsaets to include treatment time and IDs
</commit_message>
<xml_diff>
--- a/Data/Final Data/No Controls/State/STATE_NO_CONTROLS_VIC_NSW_Median_Rent.xlsx
+++ b/Data/Final Data/No Controls/State/STATE_NO_CONTROLS_VIC_NSW_Median_Rent.xlsx
@@ -361,7 +361,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -414,6 +414,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +454,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -484,6 +492,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -519,6 +530,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -554,6 +568,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -589,6 +606,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -624,6 +644,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -659,6 +682,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -694,6 +720,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -729,6 +758,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -764,6 +796,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -799,6 +834,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -834,6 +872,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -869,6 +910,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -904,6 +948,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -939,6 +986,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -974,6 +1024,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1009,6 +1062,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1044,6 +1100,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1079,6 +1138,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1114,6 +1176,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1149,6 +1214,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1184,6 +1252,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1219,6 +1290,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1254,6 +1328,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1289,6 +1366,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1324,6 +1404,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1359,6 +1442,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1394,6 +1480,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1429,6 +1518,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1464,6 +1556,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1499,6 +1594,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1534,6 +1632,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1569,6 +1670,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1604,6 +1708,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1639,6 +1746,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1674,6 +1784,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1709,6 +1822,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1743,6 +1859,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1752,7 +1871,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -1805,6 +1924,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1840,6 +1964,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1875,6 +2002,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1910,6 +2040,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1945,6 +2078,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1980,6 +2116,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2015,6 +2154,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2050,6 +2192,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2085,6 +2230,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2120,6 +2268,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2155,6 +2306,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2190,6 +2344,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2225,6 +2382,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2260,6 +2420,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2295,6 +2458,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2330,6 +2496,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2365,6 +2534,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2400,6 +2572,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2435,6 +2610,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2470,6 +2648,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2505,6 +2686,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2540,6 +2724,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2575,6 +2762,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2610,6 +2800,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2645,6 +2838,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2680,6 +2876,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2715,6 +2914,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2750,6 +2952,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2785,6 +2990,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2820,6 +3028,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2855,6 +3066,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2890,6 +3104,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2925,6 +3142,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2960,6 +3180,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2995,6 +3218,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3030,6 +3256,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3065,6 +3294,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3100,6 +3332,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3134,6 +3369,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -3143,7 +3381,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -3196,6 +3434,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3231,6 +3474,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3266,6 +3512,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3301,6 +3550,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3336,6 +3588,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3371,6 +3626,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3406,6 +3664,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3441,6 +3702,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3476,6 +3740,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3511,6 +3778,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3546,6 +3816,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3581,6 +3854,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3616,6 +3892,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3651,6 +3930,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3686,6 +3968,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3721,6 +4006,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3756,6 +4044,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3791,6 +4082,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3826,6 +4120,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3861,6 +4158,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3896,6 +4196,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3931,6 +4234,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3966,6 +4272,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4001,6 +4310,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4036,6 +4348,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4071,6 +4386,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4106,6 +4424,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4141,6 +4462,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -4176,6 +4500,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4211,6 +4538,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4246,6 +4576,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4281,6 +4614,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4316,6 +4652,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4351,6 +4690,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4386,6 +4728,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4421,6 +4766,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4456,6 +4804,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4491,6 +4842,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4525,6 +4879,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -4534,7 +4891,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -4587,6 +4944,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -4622,6 +4984,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4657,6 +5022,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4692,6 +5060,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4727,6 +5098,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4762,6 +5136,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4797,6 +5174,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4832,6 +5212,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4867,6 +5250,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4902,6 +5288,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4937,6 +5326,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4972,6 +5364,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5007,6 +5402,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5042,6 +5440,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5077,6 +5478,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5112,6 +5516,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5147,6 +5554,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5182,6 +5592,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5217,6 +5630,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5252,6 +5668,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5287,6 +5706,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5322,6 +5744,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5357,6 +5782,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5392,6 +5820,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5427,6 +5858,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5462,6 +5896,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5497,6 +5934,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5532,6 +5972,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -5567,6 +6010,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5602,6 +6048,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5637,6 +6086,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5672,6 +6124,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5707,6 +6162,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5742,6 +6200,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5777,6 +6238,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5812,6 +6276,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -5847,6 +6314,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5882,6 +6352,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5916,6 +6389,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -5925,7 +6401,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -5978,6 +6454,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -6013,6 +6494,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -6048,6 +6532,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -6083,6 +6570,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -6118,6 +6608,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -6153,6 +6646,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6188,6 +6684,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6223,6 +6722,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -6258,6 +6760,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6293,6 +6798,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6328,6 +6836,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6363,6 +6874,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6398,6 +6912,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -6433,6 +6950,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -6468,6 +6988,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -6503,6 +7026,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -6538,6 +7064,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -6573,6 +7102,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -6608,6 +7140,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -6643,6 +7178,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6678,6 +7216,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6713,6 +7254,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6748,6 +7292,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -6783,6 +7330,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -6818,6 +7368,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -6853,6 +7406,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6888,6 +7444,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6923,6 +7482,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6958,6 +7520,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6993,6 +7558,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7028,6 +7596,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7063,6 +7634,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7098,6 +7672,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7133,6 +7710,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -7168,6 +7748,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -7203,6 +7786,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -7238,6 +7824,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -7273,6 +7862,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -7307,6 +7899,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -7316,7 +7911,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -7369,6 +7964,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7404,6 +8004,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7439,6 +8042,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7474,6 +8080,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7509,6 +8118,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7544,6 +8156,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7579,6 +8194,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7614,6 +8232,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7649,6 +8270,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7684,6 +8308,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7719,6 +8346,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7754,6 +8384,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7789,6 +8422,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7824,6 +8460,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7859,6 +8498,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -7894,6 +8536,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -7929,6 +8574,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7964,6 +8612,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7999,6 +8650,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8034,6 +8688,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8069,6 +8726,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8104,6 +8764,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8139,6 +8802,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8174,6 +8840,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8209,6 +8878,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8244,6 +8916,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8279,6 +8954,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8314,6 +8992,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8349,6 +9030,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8384,6 +9068,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8419,6 +9106,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8454,6 +9144,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8489,6 +9182,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8524,6 +9220,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8559,6 +9258,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8594,6 +9296,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8629,6 +9334,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8664,6 +9372,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8698,6 +9409,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -8707,7 +9421,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="8" max="8" width="20.7109375" style="2" customWidth="1"/>
@@ -8760,6 +9474,11 @@
           <t>Quarter_End_Date</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Treated_Time</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -8795,6 +9514,9 @@
       <c r="I2" s="2">
         <v>43190</v>
       </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8830,6 +9552,9 @@
       <c r="I3" s="2">
         <v>43281</v>
       </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8865,6 +9590,9 @@
       <c r="I4" s="2">
         <v>43373</v>
       </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8900,6 +9628,9 @@
       <c r="I5" s="2">
         <v>43465</v>
       </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8935,6 +9666,9 @@
       <c r="I6" s="2">
         <v>43555</v>
       </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8970,6 +9704,9 @@
       <c r="I7" s="2">
         <v>43646</v>
       </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -9005,6 +9742,9 @@
       <c r="I8" s="2">
         <v>43738</v>
       </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -9040,6 +9780,9 @@
       <c r="I9" s="2">
         <v>43830</v>
       </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -9075,6 +9818,9 @@
       <c r="I10" s="2">
         <v>43921</v>
       </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9110,6 +9856,9 @@
       <c r="I11" s="2">
         <v>44012</v>
       </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9145,6 +9894,9 @@
       <c r="I12" s="2">
         <v>44104</v>
       </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9180,6 +9932,9 @@
       <c r="I13" s="2">
         <v>44196</v>
       </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9215,6 +9970,9 @@
       <c r="I14" s="2">
         <v>44286</v>
       </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9250,6 +10008,9 @@
       <c r="I15" s="2">
         <v>44377</v>
       </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9285,6 +10046,9 @@
       <c r="I16" s="2">
         <v>44469</v>
       </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9320,6 +10084,9 @@
       <c r="I17" s="2">
         <v>44561</v>
       </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9355,6 +10122,9 @@
       <c r="I18" s="2">
         <v>44651</v>
       </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9390,6 +10160,9 @@
       <c r="I19" s="2">
         <v>44742</v>
       </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9425,6 +10198,9 @@
       <c r="I20" s="2">
         <v>44834</v>
       </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9460,6 +10236,9 @@
       <c r="I21" s="2">
         <v>43190</v>
       </c>
+      <c r="J21">
+        <v>13</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9495,6 +10274,9 @@
       <c r="I22" s="2">
         <v>43281</v>
       </c>
+      <c r="J22">
+        <v>13</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9530,6 +10312,9 @@
       <c r="I23" s="2">
         <v>43373</v>
       </c>
+      <c r="J23">
+        <v>13</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9565,6 +10350,9 @@
       <c r="I24" s="2">
         <v>43465</v>
       </c>
+      <c r="J24">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9600,6 +10388,9 @@
       <c r="I25" s="2">
         <v>43555</v>
       </c>
+      <c r="J25">
+        <v>13</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -9635,6 +10426,9 @@
       <c r="I26" s="2">
         <v>43646</v>
       </c>
+      <c r="J26">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -9670,6 +10464,9 @@
       <c r="I27" s="2">
         <v>43738</v>
       </c>
+      <c r="J27">
+        <v>13</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9705,6 +10502,9 @@
       <c r="I28" s="2">
         <v>43830</v>
       </c>
+      <c r="J28">
+        <v>13</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9740,6 +10540,9 @@
       <c r="I29" s="2">
         <v>43921</v>
       </c>
+      <c r="J29">
+        <v>13</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9775,6 +10578,9 @@
       <c r="I30" s="2">
         <v>44012</v>
       </c>
+      <c r="J30">
+        <v>13</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9810,6 +10616,9 @@
       <c r="I31" s="2">
         <v>44104</v>
       </c>
+      <c r="J31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -9845,6 +10654,9 @@
       <c r="I32" s="2">
         <v>44196</v>
       </c>
+      <c r="J32">
+        <v>13</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9880,6 +10692,9 @@
       <c r="I33" s="2">
         <v>44286</v>
       </c>
+      <c r="J33">
+        <v>13</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9915,6 +10730,9 @@
       <c r="I34" s="2">
         <v>44377</v>
       </c>
+      <c r="J34">
+        <v>13</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9950,6 +10768,9 @@
       <c r="I35" s="2">
         <v>44469</v>
       </c>
+      <c r="J35">
+        <v>13</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9985,6 +10806,9 @@
       <c r="I36" s="2">
         <v>44561</v>
       </c>
+      <c r="J36">
+        <v>13</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -10020,6 +10844,9 @@
       <c r="I37" s="2">
         <v>44651</v>
       </c>
+      <c r="J37">
+        <v>13</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -10055,6 +10882,9 @@
       <c r="I38" s="2">
         <v>44742</v>
       </c>
+      <c r="J38">
+        <v>13</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -10089,6 +10919,9 @@
       </c>
       <c r="I39" s="2">
         <v>44834</v>
+      </c>
+      <c r="J39">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>